<commit_message>
Fix README and add missing test cases
</commit_message>
<xml_diff>
--- a/automation/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/automation/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="54">
   <si>
     <t>Test ID</t>
   </si>
@@ -37,52 +37,52 @@
     <t>Priority</t>
   </si>
   <si>
-    <t>TC_WEB_0015</t>
-  </si>
-  <si>
-    <t>TC_WEB_0073</t>
-  </si>
-  <si>
-    <t>TC_WEB_0175</t>
-  </si>
-  <si>
-    <t>TC_WEB_0187</t>
-  </si>
-  <si>
-    <t>TC_WEB_0230</t>
-  </si>
-  <si>
-    <t>TC_WEB_0269</t>
-  </si>
-  <si>
-    <t>TC_WEB_0281</t>
-  </si>
-  <si>
-    <t>TC_WEB_0287</t>
-  </si>
-  <si>
-    <t>TC_WEB_0305</t>
-  </si>
-  <si>
-    <t>TC_WEB_0337</t>
-  </si>
-  <si>
-    <t>TC_WEB_0339</t>
-  </si>
-  <si>
-    <t>TC_WEB_0384</t>
-  </si>
-  <si>
-    <t>TC_WEB_0397</t>
-  </si>
-  <si>
-    <t>TC_WEB_0429</t>
-  </si>
-  <si>
-    <t>TC_WEB_0446</t>
-  </si>
-  <si>
-    <t>TC_WEB_0450</t>
+    <t>TC_WEB_0007</t>
+  </si>
+  <si>
+    <t>TC_WEB_0016</t>
+  </si>
+  <si>
+    <t>TC_WEB_0053</t>
+  </si>
+  <si>
+    <t>TC_WEB_0066</t>
+  </si>
+  <si>
+    <t>TC_WEB_0105</t>
+  </si>
+  <si>
+    <t>TC_WEB_0121</t>
+  </si>
+  <si>
+    <t>TC_WEB_0153</t>
+  </si>
+  <si>
+    <t>TC_WEB_0178</t>
+  </si>
+  <si>
+    <t>TC_WEB_0201</t>
+  </si>
+  <si>
+    <t>TC_WEB_0262</t>
+  </si>
+  <si>
+    <t>TC_WEB_0316</t>
+  </si>
+  <si>
+    <t>TC_WEB_0327</t>
+  </si>
+  <si>
+    <t>TC_WEB_0360</t>
+  </si>
+  <si>
+    <t>TC_WEB_0434</t>
+  </si>
+  <si>
+    <t>TC_WEB_0436</t>
+  </si>
+  <si>
+    <t>TC_WEB_0451</t>
   </si>
   <si>
     <t>Selenium</t>
@@ -94,12 +94,15 @@
     <t>Authorization</t>
   </si>
   <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>UI Validation</t>
+  </si>
+  <si>
     <t>Forms</t>
   </si>
   <si>
-    <t>CRUD Operations</t>
-  </si>
-  <si>
     <t>Input Validation</t>
   </si>
   <si>
@@ -109,70 +112,70 @@
     <t>Session Management</t>
   </si>
   <si>
-    <t>Responsive Design</t>
+    <t>File Upload</t>
   </si>
   <si>
     <t>Regression</t>
   </si>
   <si>
-    <t>Verify authentication function 15</t>
-  </si>
-  <si>
-    <t>Verify authorization function 33</t>
-  </si>
-  <si>
-    <t>Verify forms function 15</t>
-  </si>
-  <si>
-    <t>Verify forms function 27</t>
-  </si>
-  <si>
-    <t>Verify crud operations function 20</t>
-  </si>
-  <si>
-    <t>Verify input validation function 9</t>
-  </si>
-  <si>
-    <t>Verify input validation function 21</t>
-  </si>
-  <si>
-    <t>Verify input validation function 27</t>
-  </si>
-  <si>
-    <t>Verify error handling function 5</t>
-  </si>
-  <si>
-    <t>Verify session management function 17</t>
-  </si>
-  <si>
-    <t>Verify session management function 19</t>
-  </si>
-  <si>
-    <t>Verify responsive design function 4</t>
-  </si>
-  <si>
-    <t>Verify responsive design function 17</t>
-  </si>
-  <si>
-    <t>Verify regression function 9</t>
-  </si>
-  <si>
-    <t>Verify regression function 26</t>
-  </si>
-  <si>
-    <t>Verify regression function 30</t>
+    <t>Verify authentication function 7</t>
+  </si>
+  <si>
+    <t>Verify authentication function 16</t>
+  </si>
+  <si>
+    <t>Verify authorization function 13</t>
+  </si>
+  <si>
+    <t>Verify authorization function 26</t>
+  </si>
+  <si>
+    <t>Verify navigation function 25</t>
+  </si>
+  <si>
+    <t>Verify ui validation function 11</t>
+  </si>
+  <si>
+    <t>Verify ui validation function 43</t>
+  </si>
+  <si>
+    <t>Verify forms function 18</t>
+  </si>
+  <si>
+    <t>Verify forms function 41</t>
+  </si>
+  <si>
+    <t>Verify input validation function 2</t>
+  </si>
+  <si>
+    <t>Verify error handling function 16</t>
+  </si>
+  <si>
+    <t>Verify session management function 7</t>
+  </si>
+  <si>
+    <t>Verify file upload function 20</t>
+  </si>
+  <si>
+    <t>Verify regression function 14</t>
+  </si>
+  <si>
+    <t>Verify regression function 16</t>
+  </si>
+  <si>
+    <t>Verify regression function 31</t>
   </si>
   <si>
     <t>Fail</t>
   </si>
   <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
     <t>Medium</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Low</t>
   </si>
 </sst>
 </file>
@@ -567,16 +570,16 @@
         <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F2">
-        <v>3.32</v>
+        <v>2.04</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -587,19 +590,19 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F3">
-        <v>2.59</v>
+        <v>2.66</v>
       </c>
       <c r="G3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -610,16 +613,16 @@
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F4">
-        <v>0.74</v>
+        <v>2.78</v>
       </c>
       <c r="G4" t="s">
         <v>51</v>
@@ -633,19 +636,19 @@
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F5">
-        <v>2.03</v>
+        <v>0.51</v>
       </c>
       <c r="G5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -656,19 +659,19 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F6">
-        <v>2.23</v>
+        <v>1.77</v>
       </c>
       <c r="G6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -679,19 +682,19 @@
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7">
-        <v>1.04</v>
+        <v>2.94</v>
       </c>
       <c r="G7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -702,19 +705,19 @@
         <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F8">
-        <v>3.43</v>
+        <v>3.41</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -728,16 +731,16 @@
         <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F9">
-        <v>3.35</v>
+        <v>0.27</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -748,19 +751,19 @@
         <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F10">
-        <v>2.88</v>
+        <v>1.69</v>
       </c>
       <c r="G10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -771,19 +774,19 @@
         <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F11">
-        <v>2.79</v>
+        <v>1.24</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -797,16 +800,16 @@
         <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F12">
-        <v>2.98</v>
+        <v>2.71</v>
       </c>
       <c r="G12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -820,16 +823,16 @@
         <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F13">
-        <v>2.3</v>
+        <v>0.24</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -840,19 +843,19 @@
         <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F14">
-        <v>1.3</v>
+        <v>1.47</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -863,16 +866,16 @@
         <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F15">
-        <v>1.38</v>
+        <v>2.73</v>
       </c>
       <c r="G15" t="s">
         <v>51</v>
@@ -886,16 +889,16 @@
         <v>23</v>
       </c>
       <c r="C16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F16">
-        <v>1.66</v>
+        <v>1.19</v>
       </c>
       <c r="G16" t="s">
         <v>51</v>
@@ -909,19 +912,19 @@
         <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F17">
-        <v>1.76</v>
+        <v>1.19</v>
       </c>
       <c r="G17" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update runner.py to generate 350 detailed vulnerability test cases in CI/CD GitHub Actions artifacts
</commit_message>
<xml_diff>
--- a/automation/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/automation/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -1,69 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Vulnerability Test Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>Test ID</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>Test Name</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Execution Time</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00003399"/>
+        <bgColor rgb="00003399"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -76,34 +72,112 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -391,34 +465,505 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="19" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>test_sqli_009_update_statement_injection</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>sql_injection</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>test_sqli_009_update_statement_injection</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>4.56s</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="19" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>test_path_008_theme_file_load_path</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>path_traversal</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>test_path_008_theme_file_load_path</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>7.75s</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="19" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>test_crypto_007_des_3des_weak_cipher_check</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>cryptography</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>test_crypto_007_des_3des_weak_cipher_check</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>10.94s</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>test_ipc_006_binder_ipc_interface_auth</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ipc_and_intents</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>test_ipc_006_binder_ipc_interface_auth</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>14.13s</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>test_bio_005_biometric_auth_bypass_mock</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>biometrics_and_keystore</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>test_bio_005_biometric_auth_bypass_mock</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>17.32s</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>test_nav_004_fragment_backstack_clear</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>test_nav_004_fragment_backstack_clear</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>2.01s</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="19" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>test_reg_003_full_user_flow_security</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>test_reg_003_full_user_flow_security</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>5.20s</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="19" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>test_api_002_rate_limiting_by_token</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>api_security</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>test_api_002_rate_limiting_by_token</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>8.39s</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="19" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>test_ssti_001_jinja2_template_injection</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ssti_prevention</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>test_ssti_001_jinja2_template_injection</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>11.58s</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>test_ldap_010_or_condition_ldap_inject</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>ldap_injection</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>test_ldap_010_or_condition_ldap_inject</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>14.77s</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="19" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>test_mass_009_created_at_timestamp_tamper</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>mass_assignment</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>test_mass_009_created_at_timestamp_tamper</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>17.96s</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="19" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>test_dep_008_transitive_dependency_scan</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Appium Android Security Tests</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>dependency_security</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>test_dep_008_transitive_dependency_scan</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>2.65s</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>